<commit_message>
feat: fixed project scores (1分/2分), PK template down to name+project columns
</commit_message>
<xml_diff>
--- a/营销PK赛模板.xlsx
+++ b/营销PK赛模板.xlsx
@@ -150,12 +150,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>必填，加分项目名称，例如：首投成功。</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>必填，本次加多少分，例如：5。可以是任意数字（可为 0）。</t>
+        <t>必填，项目名称，须为固定项目之一（分值由程序自动判定）。</t>
       </text>
     </comment>
   </commentList>
@@ -451,12 +446,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,11 +464,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>分值</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>